<commit_message>
Update weak current report metadata and sample data wording
</commit_message>
<xml_diff>
--- a/综合物理实验I+日程和教师安排循环表+20260305.xlsx
+++ b/综合物理实验I+日程和教师安排循环表+20260305.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Personal Profile\Profile\UCAS\t-Sophomore\S2\Comprehensive Physics Experiments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Personal Profile\Profile\Ucas\t-Sophomore\S2\Comprehensive Physics Experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF8D921-9334-47E6-AF46-13052255CA62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{567C4C63-3F1E-42F1-95C9-AF3C2E7A5676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1073" yWindow="1073" windowWidth="17280" windowHeight="9982" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="日程安排" sheetId="7" r:id="rId1"/>
@@ -121,83 +121,84 @@
     <t>学园二349</t>
   </si>
   <si>
+    <t>4、5</t>
+  </si>
+  <si>
+    <t>3月23、30日</t>
+  </si>
+  <si>
+    <t>布朗运动</t>
+  </si>
+  <si>
+    <t>3月25日、4月1日</t>
+  </si>
+  <si>
+    <t>学园二342</t>
+  </si>
+  <si>
+    <t>纪爱玲</t>
+  </si>
+  <si>
+    <t>4月6日（放假）</t>
+  </si>
+  <si>
+    <t>西实验楼206</t>
+  </si>
+  <si>
+    <t>王正川</t>
+  </si>
+  <si>
+    <t>7、8</t>
+  </si>
+  <si>
+    <t>4月13、20日</t>
+  </si>
+  <si>
+    <t>4月15、22日</t>
+  </si>
+  <si>
+    <t>西实验楼204</t>
+  </si>
+  <si>
+    <t>彭毅</t>
+  </si>
+  <si>
+    <t>9、11</t>
+  </si>
+  <si>
+    <t>4月27日，5月11日</t>
+  </si>
+  <si>
+    <t>4月29日，5月13日</t>
+  </si>
+  <si>
+    <t>5月4日（放假）</t>
+  </si>
+  <si>
+    <t>12、13</t>
+  </si>
+  <si>
+    <t>5月18、25日</t>
+  </si>
+  <si>
+    <t>5月20、27日</t>
+  </si>
+  <si>
+    <t>14、15</t>
+  </si>
+  <si>
+    <t>6月1日、8日</t>
+  </si>
+  <si>
+    <t>6月3日、10日</t>
+  </si>
+  <si>
+    <t>葛琛</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
     <t>马肖燕（周一）
 孟洋（周三）</t>
-  </si>
-  <si>
-    <t>4、5</t>
-  </si>
-  <si>
-    <t>3月23、30日</t>
-  </si>
-  <si>
-    <t>布朗运动</t>
-  </si>
-  <si>
-    <t>3月25日、4月1日</t>
-  </si>
-  <si>
-    <t>学园二342</t>
-  </si>
-  <si>
-    <t>纪爱玲</t>
-  </si>
-  <si>
-    <t>4月6日（放假）</t>
-  </si>
-  <si>
-    <t>西实验楼206</t>
-  </si>
-  <si>
-    <t>王正川</t>
-  </si>
-  <si>
-    <t>7、8</t>
-  </si>
-  <si>
-    <t>4月13、20日</t>
-  </si>
-  <si>
-    <t>4月15、22日</t>
-  </si>
-  <si>
-    <t>西实验楼204</t>
-  </si>
-  <si>
-    <t>彭毅</t>
-  </si>
-  <si>
-    <t>9、11</t>
-  </si>
-  <si>
-    <t>4月27日，5月11日</t>
-  </si>
-  <si>
-    <t>4月29日，5月13日</t>
-  </si>
-  <si>
-    <t>5月4日（放假）</t>
-  </si>
-  <si>
-    <t>12、13</t>
-  </si>
-  <si>
-    <t>5月18、25日</t>
-  </si>
-  <si>
-    <t>5月20、27日</t>
-  </si>
-  <si>
-    <t>14、15</t>
-  </si>
-  <si>
-    <t>6月1日、8日</t>
-  </si>
-  <si>
-    <t>6月3日、10日</t>
-  </si>
-  <si>
-    <t>葛琛</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -206,7 +207,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="178" formatCode="m&quot;月&quot;d&quot;日&quot;;@"/>
+    <numFmt numFmtId="176" formatCode="m&quot;月&quot;d&quot;日&quot;;@"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -363,7 +364,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="178" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -976,7 +977,7 @@
         <v>23</v>
       </c>
       <c r="P3" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1022,16 +1023,16 @@
         <v>31</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>27</v>
@@ -1046,10 +1047,10 @@
         <v>28</v>
       </c>
       <c r="H5" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" s="10" t="s">
         <v>35</v>
-      </c>
-      <c r="I5" s="10" t="s">
-        <v>36</v>
       </c>
       <c r="J5" s="10" t="s">
         <v>27</v>
@@ -1065,10 +1066,10 @@
         <v>26</v>
       </c>
       <c r="O5" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="P5" s="10" t="s">
         <v>37</v>
-      </c>
-      <c r="P5" s="10" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1077,7 +1078,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
@@ -1097,19 +1098,19 @@
         <v>28</v>
       </c>
       <c r="O6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="P6" s="10" t="s">
         <v>40</v>
-      </c>
-      <c r="P6" s="10" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>22</v>
@@ -1121,13 +1122,13 @@
         <v>28</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>26</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>22</v>
@@ -1140,22 +1141,22 @@
         <v>6</v>
       </c>
       <c r="N7" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O7" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="P7" s="10" t="s">
         <v>45</v>
-      </c>
-      <c r="P7" s="10" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>17</v>
@@ -1164,7 +1165,7 @@
         <v>28</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>26</v>
@@ -1173,7 +1174,7 @@
         <v>27</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>17</v>
@@ -1193,7 +1194,7 @@
         <v>10</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
@@ -1213,17 +1214,17 @@
     </row>
     <row r="10" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>28</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F10" s="10" t="s">
         <v>26</v>
@@ -1235,13 +1236,13 @@
         <v>22</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J10" s="10" t="s">
         <v>28</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
@@ -1251,14 +1252,14 @@
     </row>
     <row r="11" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="18" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>26</v>
@@ -1273,10 +1274,10 @@
         <v>17</v>
       </c>
       <c r="I11" s="18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K11" s="10" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
Add experimental report for Vacuum Preparation and Thermal Evaporation Coating
- Created a comprehensive LaTeX document detailing the objectives, instruments, principles, procedures, data processing, and analysis related to the vacuum experiment.
- Included sections on vacuum concepts, equipment descriptions, experimental methods, and results interpretation.
- Document formatted with appropriate packages for mathematical expressions, figures, and tables.
</commit_message>
<xml_diff>
--- a/综合物理实验I+日程和教师安排循环表+20260305.xlsx
+++ b/综合物理实验I+日程和教师安排循环表+20260305.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Personal Profile\Profile\Ucas\t-Sophomore\S2\Comprehensive Physics Experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{567C4C63-3F1E-42F1-95C9-AF3C2E7A5676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4EAA970-1609-4527-8946-6A5A6346FEAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="17280" windowHeight="9975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="日程安排" sheetId="7" r:id="rId1"/>
@@ -82,9 +82,6 @@
     <t>教一楼428</t>
   </si>
   <si>
-    <t>郭沁林</t>
-  </si>
-  <si>
     <t>集体讲座，真空，教一楼108</t>
   </si>
   <si>
@@ -199,6 +196,10 @@
   <si>
     <t>马肖燕（周一）
 孟洋（周三）</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>郭沁林</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -941,7 +942,7 @@
         <v>18</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>19</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:16" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -953,7 +954,7 @@
         <v>46083</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E3" s="27"/>
       <c r="F3" s="27"/>
@@ -963,7 +964,7 @@
         <v>46085</v>
       </c>
       <c r="J3" s="29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K3" s="30"/>
       <c r="L3" s="9"/>
@@ -971,105 +972,105 @@
         <v>2</v>
       </c>
       <c r="N3" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="O3" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="O3" s="10" t="s">
-        <v>23</v>
-      </c>
       <c r="P3" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>27</v>
-      </c>
       <c r="F4" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>17</v>
       </c>
       <c r="H4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="I4" s="10" t="s">
-        <v>29</v>
-      </c>
       <c r="J4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="K4" s="10" t="s">
         <v>26</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>27</v>
       </c>
       <c r="L4" s="6"/>
       <c r="M4" s="10">
         <v>3</v>
       </c>
       <c r="N4" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="O4" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="O4" s="10" t="s">
-        <v>31</v>
-      </c>
       <c r="P4" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H5" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="10" t="s">
-        <v>35</v>
-      </c>
       <c r="J5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L5" s="6"/>
       <c r="M5" s="10">
         <v>4</v>
       </c>
       <c r="N5" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O5" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="P5" s="10" t="s">
         <v>36</v>
-      </c>
-      <c r="P5" s="10" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1078,7 +1079,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
@@ -1095,43 +1096,43 @@
         <v>5</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O6" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="P6" s="10" t="s">
         <v>39</v>
-      </c>
-      <c r="P6" s="10" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>17</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>17</v>
@@ -1141,46 +1142,46 @@
         <v>6</v>
       </c>
       <c r="N7" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O7" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="P7" s="10" t="s">
         <v>44</v>
-      </c>
-      <c r="P7" s="10" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>17</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G8" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="10" t="s">
-        <v>27</v>
-      </c>
       <c r="I8" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>17</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L8" s="6"/>
       <c r="M8" s="15"/>
@@ -1194,7 +1195,7 @@
         <v>10</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
@@ -1214,35 +1215,35 @@
     </row>
     <row r="10" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="I10" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G10" s="10" t="s">
+      <c r="J10" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="H10" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="I10" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="J10" s="10" t="s">
-        <v>28</v>
-      </c>
       <c r="K10" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
@@ -1252,35 +1253,35 @@
     </row>
     <row r="11" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E11" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>27</v>
-      </c>
       <c r="G11" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>17</v>
       </c>
       <c r="I11" s="18" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>

</xml_diff>